<commit_message>
Atualiza exemplo de saldo pra refletir melhor o formato real
config/saldos.example.xlsx agora tem 26 linhas divididas entre 3
bankers fictícios (18/5/3), espelhando a distribuição e os valores
(incluindo saldos negativos e centavos) de uma planilha real de saldo
em conta do escritório inteiro. Antes o exemplo tinha só 3 linhas e 2
bankers, o que não representava bem o volume/variedade de um export
de verdade. Nomes de cliente e conta continuam fictícios/genéricos.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QWgeXNNmjYVnh184fZ5Ac9
</commit_message>
<xml_diff>
--- a/config/saldos.example.xlsx
+++ b/config/saldos.example.xlsx
@@ -413,8 +413,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -441,16 +447,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>001111111</t>
+          <t>000100001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ABC_XY</t>
+          <t>CLI_100001</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>12345.67</v>
+        <v>-5225.7</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -461,16 +467,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>002222222</t>
+          <t>000100002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DEF_ZW</t>
+          <t>CLI_100002</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>890.1</v>
+        <v>106.77</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -481,20 +487,480 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>003333333</t>
+          <t>000100003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GHI_QR</t>
+          <t>CLI_100003</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-250</v>
+        <v>0.36</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>000100004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CLI_100004</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>98.56</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>000100005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CLI_100005</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>000100006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CLI_100006</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>000100007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CLI_100007</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>000100008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CLI_100008</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>000100009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CLI_100009</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>000100010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CLI_100010</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>7870.74</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>000100011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CLI_100011</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>23810.86</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>000100012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CLI_100012</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>000100013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CLI_100013</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>000100014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CLI_100014</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1287.81</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>000100015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CLI_100015</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>462.72</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>000100016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CLI_100016</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>000100017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CLI_100017</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>577.89</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>000100018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CLI_100018</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>559.3</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Fulano Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>000100019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CLI_100019</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>Beltrano Souza</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>000100020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CLI_100020</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Beltrano Souza</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>000100021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CLI_100021</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1003.98</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Beltrano Souza</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>000100022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CLI_100022</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>6285.02</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Beltrano Souza</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>000100023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CLI_100023</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3037.88</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Beltrano Souza</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>000100024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CLI_100024</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Ciclano Nunes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>000100025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CLI_100025</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>-492.32</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Ciclano Nunes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>000100026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CLI_100026</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Ciclano Nunes</t>
         </is>
       </c>
     </row>

</xml_diff>